<commit_message>
Add OOTB vs proposal workflow comparison sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018d6Sqji3PhM1w1Xd54RvCw
</commit_message>
<xml_diff>
--- a/docs/moc/Impala - MOC Workflow Variants (Full - Emergency - Simple).xlsx
+++ b/docs/moc/Impala - MOC Workflow Variants (Full - Emergency - Simple).xlsx
@@ -7,10 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Full MOC" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Emergency" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. Simple" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparison" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Full MOC" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Emergency" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. Simple" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,8 +44,12 @@
       <i val="1"/>
       <color rgb="007F7F7F"/>
     </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00595959"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -69,6 +74,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00BDD7EE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
   </fills>
@@ -98,14 +113,35 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -122,17 +158,10 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -590,6 +619,521 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>MOC workflows - Intelex out of the box vs Impala proposal</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Out of the Box (Intelex)</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n"/>
+      <c r="C3" s="3" t="n"/>
+      <c r="D3" s="3" t="n"/>
+      <c r="E3" s="3" t="n"/>
+    </row>
+    <row r="4" ht="46" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Stage #</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Stage Name</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Replacement in Kind
+(Replacement in Kind = Yes)</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Emergency
+(Emergency Change = Yes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Initiation</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Pre-Approval</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Evaluation</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Design &amp; Analysis</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Implementation</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Start Up</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Follow Up</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="n"/>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Path (stage #)</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>1-2-3-4-5-6-7</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>1-2-5-6-7</t>
+        </is>
+      </c>
+      <c r="E12" s="10" t="inlineStr">
+        <is>
+          <t>1-2-4-5-6-7</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>Replacement in Kind skips Evaluation and Design &amp; Analysis; Emergency skips Evaluation (both decided at Pre-Approval).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Proposal (Impala - MOC Proposal Rev2)</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n"/>
+      <c r="C15" s="3" t="n"/>
+      <c r="D15" s="3" t="n"/>
+      <c r="E15" s="3" t="n"/>
+    </row>
+    <row r="16" ht="46" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Stage #</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Stage Name</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Simple
+(Simple Change = Yes)</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Emergency
+(Emergency Change = Yes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Initiation</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Evaluation, Design &amp; Analysis</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="D18" s="12" t="inlineStr">
+        <is>
+          <t>✔ no checklist</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Approval</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Implementation</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Start Up</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Follow Up</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="n"/>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>Path (stage #)</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="inlineStr">
+        <is>
+          <t>1-2-3-4-5-6</t>
+        </is>
+      </c>
+      <c r="D23" s="10" t="inlineStr">
+        <is>
+          <t>1-2-3-4-5-6</t>
+        </is>
+      </c>
+      <c r="E23" s="10" t="inlineStr">
+        <is>
+          <t>1-3-4-5-6</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t>Simple (replaces Replacement in Kind, for IT / organisational changes) keeps all stages but no Evaluation, D&amp;A checklist; Emergency goes straight from Initiation to Approval.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="13" t="inlineStr">
+        <is>
+          <t>Legend:</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>✔ stage applies</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>— stage skipped</t>
+        </is>
+      </c>
+      <c r="D26" s="12" t="inlineStr">
+        <is>
+          <t>applies with differences</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -609,281 +1153,281 @@
       </c>
     </row>
     <row r="2" ht="32" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>Intelex configures ONE MOC workflow; the Emergency and Simple variants are paths/rules driven by the Initiation flags. Not three separate workflows (keeps the change within SOW 'Moderate configuration').</t>
         </is>
       </c>
     </row>
     <row r="4" ht="36" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Stage #</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Stage Name</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Full MOC
 (Emergency = No, Simple = No)</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Emergency
 (Emergency Change = Yes)</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>Simple
 (Simple Change = Yes)</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="5" ht="34" customHeight="1">
-      <c r="A5" s="4" t="n">
+      <c r="A5" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="16" t="inlineStr">
         <is>
           <t>Initiation</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="16" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="16" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E5" s="16" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="F5" s="16" t="inlineStr">
         <is>
           <t>Emergency: Emergency Justification [BA]. Simple: Change Type typically 4 (IT) or 5 (Org).</t>
         </is>
       </c>
     </row>
     <row r="6" ht="34" customHeight="1">
-      <c r="A6" s="4" t="n">
+      <c r="A6" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="16" t="inlineStr">
         <is>
           <t>Evaluation, Design &amp; Analysis</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="16" t="inlineStr">
         <is>
           <t>Yes - checklist + tasks + D&amp;A questions</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D6" s="17" t="inlineStr">
         <is>
           <t>SKIPPED - straight to Approval</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr">
+      <c r="E6" s="18" t="inlineStr">
         <is>
           <t>Yes - NO checklist (tasks + D&amp;A questions [TBC which])</t>
         </is>
       </c>
-      <c r="F6" s="7" t="inlineStr">
+      <c r="F6" s="18" t="inlineStr">
         <is>
           <t>Emergency: retrospective completion? [TBC]. Simple: 'different process review' [TBC].</t>
         </is>
       </c>
     </row>
     <row r="7" ht="34" customHeight="1">
-      <c r="A7" s="4" t="n">
+      <c r="A7" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="16" t="inlineStr">
         <is>
           <t>Approval</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C7" s="16" t="inlineStr">
         <is>
           <t>Yes - sequential by Change Impact</t>
         </is>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="D7" s="18" t="inlineStr">
         <is>
           <t>Yes - who approves an emergency? [TBC]</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E7" s="16" t="inlineStr">
         <is>
           <t>Yes - sequential by Change Impact</t>
         </is>
       </c>
-      <c r="F7" s="7" t="inlineStr">
+      <c r="F7" s="18" t="inlineStr">
         <is>
           <t>Due 7 days (emergency due date [TBC]).</t>
         </is>
       </c>
     </row>
     <row r="8" ht="34" customHeight="1">
-      <c r="A8" s="4" t="n">
+      <c r="A8" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="16" t="inlineStr">
         <is>
           <t>Implementation</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" s="16" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="16" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr">
+      <c r="E8" s="18" t="inlineStr">
         <is>
           <t>Yes - PSSR applicable? [TBC]</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="F8" s="16" t="inlineStr">
         <is>
           <t>Entry only when Pre-Implementation tasks are closed.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1">
-      <c r="A9" s="4" t="n">
+      <c r="A9" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="16" t="inlineStr">
         <is>
           <t>Start Up</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C9" s="16" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D9" s="16" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr">
+      <c r="E9" s="18" t="inlineStr">
         <is>
           <t>Yes - applicable? [TBC]</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr"/>
+      <c r="F9" s="16" t="inlineStr"/>
     </row>
     <row r="10" ht="34" customHeight="1">
-      <c r="A10" s="4" t="n">
+      <c r="A10" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="16" t="inlineStr">
         <is>
           <t>Follow Up</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C10" s="16" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D10" s="18" t="inlineStr">
         <is>
           <t>Yes - close only when regularised [TBC]</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="E10" s="16" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="F10" s="16" t="inlineStr">
         <is>
           <t>Entry only when Pre-Follow Up tasks are closed.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t>Open questions for the team</t>
         </is>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" s="14" t="inlineStr">
         <is>
           <t>1. Emergency: who approves (Change Impact matrix as normal, or a single senior approver as in BRD RULE-B3-14)?</t>
         </is>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" s="14" t="inlineStr">
         <is>
           <t>2. Emergency: is the Evaluation, D&amp;A checklist completed retrospectively? Within how many days? Can the MOC close before?</t>
         </is>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="A15" s="14" t="inlineStr">
         <is>
           <t>3. Emergency: approval due date (shorter than 7 days?).</t>
         </is>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="A16" s="14" t="inlineStr">
         <is>
           <t>4. Simple: what is the 'different process review' for IT / organisational changes - does anything need capturing in Intelex?</t>
         </is>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" s="14" t="inlineStr">
         <is>
           <t>5. Simple: which D&amp;A and Implementation questions apply (alternatives, hazard assessment, PSSR, Start Up)?</t>
         </is>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="A18" s="14" t="inlineStr">
         <is>
           <t>6. Simple: confirm it keeps all 6 stages (Rev2) rather than skipping stages like the old 'Replacement in Kind'.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="A19" s="14" t="inlineStr">
         <is>
           <t>7. If both Emergency and Simple are Yes: which rule prevails (proposal: Emergency path, no checklist)?</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="9" t="inlineStr">
+      <c r="A21" s="20" t="inlineStr">
         <is>
           <t>Legend: grey = stage skipped; yellow = to be confirmed [TBC]; [BA] = BA proposal, not in Sam's Rev2.</t>
         </is>
@@ -904,7 +1448,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -932,214 +1476,214 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="21" t="inlineStr">
         <is>
           <t>Proposal</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Stage #</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Stage Name</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>In this variant</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="n">
+      <c r="A5" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>Initiation</t>
         </is>
       </c>
-      <c r="C5" s="11" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="n">
+      <c r="A6" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="11" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Evaluation, Design &amp; Analysis</t>
         </is>
       </c>
-      <c r="C6" s="11" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="n">
+      <c r="A7" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Approval</t>
         </is>
       </c>
-      <c r="C7" s="11" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="n">
+      <c r="A8" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Implementation</t>
         </is>
       </c>
-      <c r="C8" s="11" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="n">
+      <c r="A9" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>Start Up</t>
         </is>
       </c>
-      <c r="C9" s="11" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="n">
+      <c r="A10" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>Follow Up</t>
         </is>
       </c>
-      <c r="C10" s="11" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="inlineStr">
+      <c r="A12" s="13" t="inlineStr">
         <is>
           <t>Detailed workflow (Intelex workbook format)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="13" t="inlineStr">
+      <c r="A13" s="22" t="inlineStr">
         <is>
           <t>Stage #</t>
         </is>
       </c>
-      <c r="B13" s="13" t="inlineStr">
+      <c r="B13" s="22" t="inlineStr">
         <is>
           <t>Stage Name</t>
         </is>
       </c>
-      <c r="C13" s="13" t="inlineStr">
+      <c r="C13" s="22" t="inlineStr">
         <is>
           <t>Record Status</t>
         </is>
       </c>
-      <c r="D13" s="13" t="inlineStr">
+      <c r="D13" s="22" t="inlineStr">
         <is>
           <t>Stage Owner</t>
         </is>
       </c>
-      <c r="E13" s="13" t="inlineStr">
+      <c r="E13" s="22" t="inlineStr">
         <is>
           <t>Due Date</t>
         </is>
       </c>
-      <c r="F13" s="13" t="inlineStr">
+      <c r="F13" s="22" t="inlineStr">
         <is>
           <t>Workflow Buttons</t>
         </is>
       </c>
-      <c r="G13" s="13" t="inlineStr">
+      <c r="G13" s="22" t="inlineStr">
         <is>
           <t>Workflow Path</t>
         </is>
       </c>
-      <c r="H13" s="13" t="inlineStr">
+      <c r="H13" s="22" t="inlineStr">
         <is>
           <t>Email Template #</t>
         </is>
       </c>
-      <c r="I13" s="13" t="inlineStr">
+      <c r="I13" s="22" t="inlineStr">
         <is>
           <t>Comments</t>
         </is>
       </c>
     </row>
     <row r="14" ht="60" customHeight="1">
-      <c r="A14" s="5" t="n">
+      <c r="A14" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B14" s="16" t="inlineStr">
         <is>
           <t>Initiation</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C14" s="16" t="inlineStr">
         <is>
           <t>Initiation</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D14" s="16" t="inlineStr">
         <is>
           <t>Created By (Field)</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E14" s="16" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="F14" s="16" t="inlineStr">
         <is>
           <t>Submit</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr">
+      <c r="G14" s="16" t="inlineStr">
         <is>
           <t>If 'Emergency Change' = Yes: to 'Approval'
 Else: to 'Evaluation, Design &amp; Analysis'</t>
         </is>
       </c>
-      <c r="H14" s="5" t="inlineStr">
+      <c r="H14" s="16" t="inlineStr">
         <is>
           <t>N01</t>
         </is>
       </c>
-      <c r="I14" s="5" t="inlineStr">
+      <c r="I14" s="16" t="inlineStr">
         <is>
           <t>Recipient(s): Change Requester
 Mandatory: Location, Description, Emergency, Simple, Temporary, Change Type, Change Impact, Priority, Change Justification, Requested Change Date.</t>
@@ -1147,45 +1691,45 @@
       </c>
     </row>
     <row r="15" ht="60" customHeight="1">
-      <c r="A15" s="5" t="n">
+      <c r="A15" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B15" s="16" t="inlineStr">
         <is>
           <t>Evaluation, Design &amp; Analysis</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C15" s="16" t="inlineStr">
         <is>
           <t>Evaluation, Design &amp; Analysis</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D15" s="16" t="inlineStr">
         <is>
           <t>MOC Coordinator (Role)</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="E15" s="16" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="F15" s="16" t="inlineStr">
         <is>
           <t>Submit</t>
         </is>
       </c>
-      <c r="G15" s="5" t="inlineStr">
+      <c r="G15" s="16" t="inlineStr">
         <is>
           <t>To 'Approval'</t>
         </is>
       </c>
-      <c r="H15" s="5" t="inlineStr">
+      <c r="H15" s="16" t="inlineStr">
         <is>
           <t>N01</t>
         </is>
       </c>
-      <c r="I15" s="5" t="inlineStr">
+      <c r="I15" s="16" t="inlineStr">
         <is>
           <t>Recipient(s): Change Requester
 Checklist answered (not for Simple Change), D&amp;A questions + justifications, documents attached.</t>
@@ -1193,95 +1737,95 @@
       </c>
     </row>
     <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="5" t="n"/>
-      <c r="B16" s="5" t="n"/>
-      <c r="C16" s="5" t="n"/>
-      <c r="D16" s="5" t="n"/>
-      <c r="E16" s="5" t="n"/>
-      <c r="F16" s="5" t="inlineStr">
+      <c r="A16" s="16" t="n"/>
+      <c r="B16" s="16" t="n"/>
+      <c r="C16" s="16" t="n"/>
+      <c r="D16" s="16" t="n"/>
+      <c r="E16" s="16" t="n"/>
+      <c r="F16" s="16" t="inlineStr">
         <is>
           <t>Roll Back</t>
         </is>
       </c>
-      <c r="G16" s="5" t="inlineStr">
+      <c r="G16" s="16" t="inlineStr">
         <is>
           <t>Back to 'Initiation'</t>
         </is>
       </c>
-      <c r="H16" s="5" t="inlineStr">
+      <c r="H16" s="16" t="inlineStr">
         <is>
           <t>N02</t>
         </is>
       </c>
-      <c r="I16" s="5" t="inlineStr">
+      <c r="I16" s="16" t="inlineStr">
         <is>
           <t>Recipient(s): Change Requester</t>
         </is>
       </c>
     </row>
     <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="5" t="n"/>
-      <c r="B17" s="5" t="n"/>
-      <c r="C17" s="5" t="n"/>
-      <c r="D17" s="5" t="n"/>
-      <c r="E17" s="5" t="n"/>
-      <c r="F17" s="5" t="inlineStr">
+      <c r="A17" s="16" t="n"/>
+      <c r="B17" s="16" t="n"/>
+      <c r="C17" s="16" t="n"/>
+      <c r="D17" s="16" t="n"/>
+      <c r="E17" s="16" t="n"/>
+      <c r="F17" s="16" t="inlineStr">
         <is>
           <t>Cancel</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr"/>
-      <c r="H17" s="5" t="inlineStr">
+      <c r="G17" s="16" t="inlineStr"/>
+      <c r="H17" s="16" t="inlineStr">
         <is>
           <t>N03</t>
         </is>
       </c>
-      <c r="I17" s="5" t="inlineStr">
+      <c r="I17" s="16" t="inlineStr">
         <is>
           <t>Recipient(s): Change Requester</t>
         </is>
       </c>
     </row>
     <row r="18" ht="60" customHeight="1">
-      <c r="A18" s="5" t="n">
+      <c r="A18" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B18" s="16" t="inlineStr">
         <is>
           <t>Approval</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="C18" s="16" t="inlineStr">
         <is>
           <t>Approval</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="D18" s="16" t="inlineStr">
         <is>
           <t>MOC Coordinator (Role)</t>
         </is>
       </c>
-      <c r="E18" s="5" t="inlineStr">
+      <c r="E18" s="16" t="inlineStr">
         <is>
           <t>7 days</t>
         </is>
       </c>
-      <c r="F18" s="5" t="inlineStr">
+      <c r="F18" s="16" t="inlineStr">
         <is>
           <t>Submit</t>
         </is>
       </c>
-      <c r="G18" s="5" t="inlineStr">
+      <c r="G18" s="16" t="inlineStr">
         <is>
           <t>To 'Implementation'</t>
         </is>
       </c>
-      <c r="H18" s="5" t="inlineStr">
+      <c r="H18" s="16" t="inlineStr">
         <is>
           <t>N01 / N08</t>
         </is>
       </c>
-      <c r="I18" s="5" t="inlineStr">
+      <c r="I18" s="16" t="inlineStr">
         <is>
           <t>Recipient(s): Change Requester
 Mandated approvals by Change Impact, sequential Local &gt; Regional &gt; Global; ad hoc approvals allowed.</t>
@@ -1289,96 +1833,96 @@
       </c>
     </row>
     <row r="19" ht="45" customHeight="1">
-      <c r="A19" s="5" t="n"/>
-      <c r="B19" s="5" t="n"/>
-      <c r="C19" s="5" t="n"/>
-      <c r="D19" s="5" t="n"/>
-      <c r="E19" s="5" t="n"/>
-      <c r="F19" s="5" t="inlineStr">
+      <c r="A19" s="16" t="n"/>
+      <c r="B19" s="16" t="n"/>
+      <c r="C19" s="16" t="n"/>
+      <c r="D19" s="16" t="n"/>
+      <c r="E19" s="16" t="n"/>
+      <c r="F19" s="16" t="inlineStr">
         <is>
           <t>Roll Back</t>
         </is>
       </c>
-      <c r="G19" s="5" t="inlineStr">
+      <c r="G19" s="16" t="inlineStr">
         <is>
           <t>If Emergency = Yes: back to 'Initiation'
 Else: back to 'Evaluation, Design &amp; Analysis'</t>
         </is>
       </c>
-      <c r="H19" s="5" t="inlineStr">
+      <c r="H19" s="16" t="inlineStr">
         <is>
           <t>N02</t>
         </is>
       </c>
-      <c r="I19" s="5" t="inlineStr">
+      <c r="I19" s="16" t="inlineStr">
         <is>
           <t>Recipient(s): Change Requester</t>
         </is>
       </c>
     </row>
     <row r="20" ht="16" customHeight="1">
-      <c r="A20" s="5" t="n"/>
-      <c r="B20" s="5" t="n"/>
-      <c r="C20" s="5" t="n"/>
-      <c r="D20" s="5" t="n"/>
-      <c r="E20" s="5" t="n"/>
-      <c r="F20" s="5" t="inlineStr">
+      <c r="A20" s="16" t="n"/>
+      <c r="B20" s="16" t="n"/>
+      <c r="C20" s="16" t="n"/>
+      <c r="D20" s="16" t="n"/>
+      <c r="E20" s="16" t="n"/>
+      <c r="F20" s="16" t="inlineStr">
         <is>
           <t>Cancel</t>
         </is>
       </c>
-      <c r="G20" s="5" t="inlineStr"/>
-      <c r="H20" s="5" t="inlineStr">
+      <c r="G20" s="16" t="inlineStr"/>
+      <c r="H20" s="16" t="inlineStr">
         <is>
           <t>N03</t>
         </is>
       </c>
-      <c r="I20" s="5" t="inlineStr">
+      <c r="I20" s="16" t="inlineStr">
         <is>
           <t>Recipient(s): Change Requester</t>
         </is>
       </c>
     </row>
     <row r="21" ht="60" customHeight="1">
-      <c r="A21" s="5" t="n">
+      <c r="A21" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="B21" s="16" t="inlineStr">
         <is>
           <t>Implementation</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="C21" s="16" t="inlineStr">
         <is>
           <t>Implementation</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="D21" s="16" t="inlineStr">
         <is>
           <t>MOC Coordinator (Role)</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr">
+      <c r="E21" s="16" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="F21" s="5" t="inlineStr">
+      <c r="F21" s="16" t="inlineStr">
         <is>
           <t>Submit</t>
         </is>
       </c>
-      <c r="G21" s="5" t="inlineStr">
+      <c r="G21" s="16" t="inlineStr">
         <is>
           <t>To 'Start Up'</t>
         </is>
       </c>
-      <c r="H21" s="5" t="inlineStr">
+      <c r="H21" s="16" t="inlineStr">
         <is>
           <t>N01</t>
         </is>
       </c>
-      <c r="I21" s="5" t="inlineStr">
+      <c r="I21" s="16" t="inlineStr">
         <is>
           <t>Recipient(s): Change Requester
 Entry only with Pre-Implementation tasks closed. PSSR, training, comms, installation, critical PSSR items.</t>
@@ -1386,95 +1930,95 @@
       </c>
     </row>
     <row r="22" ht="16" customHeight="1">
-      <c r="A22" s="5" t="n"/>
-      <c r="B22" s="5" t="n"/>
-      <c r="C22" s="5" t="n"/>
-      <c r="D22" s="5" t="n"/>
-      <c r="E22" s="5" t="n"/>
-      <c r="F22" s="5" t="inlineStr">
+      <c r="A22" s="16" t="n"/>
+      <c r="B22" s="16" t="n"/>
+      <c r="C22" s="16" t="n"/>
+      <c r="D22" s="16" t="n"/>
+      <c r="E22" s="16" t="n"/>
+      <c r="F22" s="16" t="inlineStr">
         <is>
           <t>Roll Back</t>
         </is>
       </c>
-      <c r="G22" s="5" t="inlineStr">
+      <c r="G22" s="16" t="inlineStr">
         <is>
           <t>Back to 'Approval'</t>
         </is>
       </c>
-      <c r="H22" s="5" t="inlineStr">
+      <c r="H22" s="16" t="inlineStr">
         <is>
           <t>N02</t>
         </is>
       </c>
-      <c r="I22" s="5" t="inlineStr">
+      <c r="I22" s="16" t="inlineStr">
         <is>
           <t>Recipient(s): Change Requester</t>
         </is>
       </c>
     </row>
     <row r="23" ht="16" customHeight="1">
-      <c r="A23" s="5" t="n"/>
-      <c r="B23" s="5" t="n"/>
-      <c r="C23" s="5" t="n"/>
-      <c r="D23" s="5" t="n"/>
-      <c r="E23" s="5" t="n"/>
-      <c r="F23" s="5" t="inlineStr">
+      <c r="A23" s="16" t="n"/>
+      <c r="B23" s="16" t="n"/>
+      <c r="C23" s="16" t="n"/>
+      <c r="D23" s="16" t="n"/>
+      <c r="E23" s="16" t="n"/>
+      <c r="F23" s="16" t="inlineStr">
         <is>
           <t>Cancel</t>
         </is>
       </c>
-      <c r="G23" s="5" t="inlineStr"/>
-      <c r="H23" s="5" t="inlineStr">
+      <c r="G23" s="16" t="inlineStr"/>
+      <c r="H23" s="16" t="inlineStr">
         <is>
           <t>N03</t>
         </is>
       </c>
-      <c r="I23" s="5" t="inlineStr">
+      <c r="I23" s="16" t="inlineStr">
         <is>
           <t>Recipient(s): Change Requester</t>
         </is>
       </c>
     </row>
     <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="5" t="n">
+      <c r="A24" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="B24" s="5" t="inlineStr">
+      <c r="B24" s="16" t="inlineStr">
         <is>
           <t>Start Up</t>
         </is>
       </c>
-      <c r="C24" s="5" t="inlineStr">
+      <c r="C24" s="16" t="inlineStr">
         <is>
           <t>Start Up</t>
         </is>
       </c>
-      <c r="D24" s="5" t="inlineStr">
+      <c r="D24" s="16" t="inlineStr">
         <is>
           <t>MOC Coordinator (Role)</t>
         </is>
       </c>
-      <c r="E24" s="5" t="inlineStr">
+      <c r="E24" s="16" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="F24" s="5" t="inlineStr">
+      <c r="F24" s="16" t="inlineStr">
         <is>
           <t>Submit</t>
         </is>
       </c>
-      <c r="G24" s="5" t="inlineStr">
+      <c r="G24" s="16" t="inlineStr">
         <is>
           <t>To 'Follow Up'</t>
         </is>
       </c>
-      <c r="H24" s="5" t="inlineStr">
+      <c r="H24" s="16" t="inlineStr">
         <is>
           <t>N01</t>
         </is>
       </c>
-      <c r="I24" s="5" t="inlineStr">
+      <c r="I24" s="16" t="inlineStr">
         <is>
           <t>Recipient(s): Change Requester
 Start-up completed, notes.</t>
@@ -1482,91 +2026,91 @@
       </c>
     </row>
     <row r="25" ht="16" customHeight="1">
-      <c r="A25" s="5" t="n"/>
-      <c r="B25" s="5" t="n"/>
-      <c r="C25" s="5" t="n"/>
-      <c r="D25" s="5" t="n"/>
-      <c r="E25" s="5" t="n"/>
-      <c r="F25" s="5" t="inlineStr">
+      <c r="A25" s="16" t="n"/>
+      <c r="B25" s="16" t="n"/>
+      <c r="C25" s="16" t="n"/>
+      <c r="D25" s="16" t="n"/>
+      <c r="E25" s="16" t="n"/>
+      <c r="F25" s="16" t="inlineStr">
         <is>
           <t>Roll Back</t>
         </is>
       </c>
-      <c r="G25" s="5" t="inlineStr">
+      <c r="G25" s="16" t="inlineStr">
         <is>
           <t>Back to 'Implementation'</t>
         </is>
       </c>
-      <c r="H25" s="5" t="inlineStr">
+      <c r="H25" s="16" t="inlineStr">
         <is>
           <t>N02</t>
         </is>
       </c>
-      <c r="I25" s="5" t="inlineStr">
+      <c r="I25" s="16" t="inlineStr">
         <is>
           <t>Recipient(s): Change Requester</t>
         </is>
       </c>
     </row>
     <row r="26" ht="16" customHeight="1">
-      <c r="A26" s="5" t="n"/>
-      <c r="B26" s="5" t="n"/>
-      <c r="C26" s="5" t="n"/>
-      <c r="D26" s="5" t="n"/>
-      <c r="E26" s="5" t="n"/>
-      <c r="F26" s="5" t="inlineStr">
+      <c r="A26" s="16" t="n"/>
+      <c r="B26" s="16" t="n"/>
+      <c r="C26" s="16" t="n"/>
+      <c r="D26" s="16" t="n"/>
+      <c r="E26" s="16" t="n"/>
+      <c r="F26" s="16" t="inlineStr">
         <is>
           <t>Cancel</t>
         </is>
       </c>
-      <c r="G26" s="5" t="inlineStr"/>
-      <c r="H26" s="5" t="inlineStr">
+      <c r="G26" s="16" t="inlineStr"/>
+      <c r="H26" s="16" t="inlineStr">
         <is>
           <t>N03</t>
         </is>
       </c>
-      <c r="I26" s="5" t="inlineStr">
+      <c r="I26" s="16" t="inlineStr">
         <is>
           <t>Recipient(s): Change Requester</t>
         </is>
       </c>
     </row>
     <row r="27" ht="45" customHeight="1">
-      <c r="A27" s="5" t="n">
+      <c r="A27" s="16" t="n">
         <v>6</v>
       </c>
-      <c r="B27" s="5" t="inlineStr">
+      <c r="B27" s="16" t="inlineStr">
         <is>
           <t>Follow Up</t>
         </is>
       </c>
-      <c r="C27" s="5" t="inlineStr">
+      <c r="C27" s="16" t="inlineStr">
         <is>
           <t>Follow Up</t>
         </is>
       </c>
-      <c r="D27" s="5" t="inlineStr">
+      <c r="D27" s="16" t="inlineStr">
         <is>
           <t>MOC Coordinator (Role)</t>
         </is>
       </c>
-      <c r="E27" s="5" t="inlineStr">
+      <c r="E27" s="16" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="F27" s="5" t="inlineStr">
+      <c r="F27" s="16" t="inlineStr">
         <is>
           <t>Close</t>
         </is>
       </c>
-      <c r="G27" s="5" t="inlineStr"/>
-      <c r="H27" s="5" t="inlineStr">
+      <c r="G27" s="16" t="inlineStr"/>
+      <c r="H27" s="16" t="inlineStr">
         <is>
           <t>N04</t>
         </is>
       </c>
-      <c r="I27" s="5" t="inlineStr">
+      <c r="I27" s="16" t="inlineStr">
         <is>
           <t>Recipient(s): Change Requester
 Entry only with Pre-Follow Up tasks closed. Temporary -&gt; permanent MOC; Lessons Learnt.</t>
@@ -1574,57 +2118,57 @@
       </c>
     </row>
     <row r="28" ht="16" customHeight="1">
-      <c r="A28" s="5" t="n"/>
-      <c r="B28" s="5" t="n"/>
-      <c r="C28" s="5" t="n"/>
-      <c r="D28" s="5" t="n"/>
-      <c r="E28" s="5" t="n"/>
-      <c r="F28" s="5" t="inlineStr">
+      <c r="A28" s="16" t="n"/>
+      <c r="B28" s="16" t="n"/>
+      <c r="C28" s="16" t="n"/>
+      <c r="D28" s="16" t="n"/>
+      <c r="E28" s="16" t="n"/>
+      <c r="F28" s="16" t="inlineStr">
         <is>
           <t>Roll Back</t>
         </is>
       </c>
-      <c r="G28" s="5" t="inlineStr">
+      <c r="G28" s="16" t="inlineStr">
         <is>
           <t>Back to 'Start Up'</t>
         </is>
       </c>
-      <c r="H28" s="5" t="inlineStr">
+      <c r="H28" s="16" t="inlineStr">
         <is>
           <t>N02</t>
         </is>
       </c>
-      <c r="I28" s="5" t="inlineStr">
+      <c r="I28" s="16" t="inlineStr">
         <is>
           <t>Recipient(s): Change Requester</t>
         </is>
       </c>
     </row>
     <row r="29" ht="16" customHeight="1">
-      <c r="A29" s="5" t="n"/>
-      <c r="B29" s="5" t="n"/>
-      <c r="C29" s="5" t="n"/>
-      <c r="D29" s="5" t="n"/>
-      <c r="E29" s="5" t="n"/>
-      <c r="F29" s="5" t="inlineStr">
+      <c r="A29" s="16" t="n"/>
+      <c r="B29" s="16" t="n"/>
+      <c r="C29" s="16" t="n"/>
+      <c r="D29" s="16" t="n"/>
+      <c r="E29" s="16" t="n"/>
+      <c r="F29" s="16" t="inlineStr">
         <is>
           <t>Cancel</t>
         </is>
       </c>
-      <c r="G29" s="5" t="inlineStr"/>
-      <c r="H29" s="5" t="inlineStr">
+      <c r="G29" s="16" t="inlineStr"/>
+      <c r="H29" s="16" t="inlineStr">
         <is>
           <t>N03</t>
         </is>
       </c>
-      <c r="I29" s="5" t="inlineStr">
+      <c r="I29" s="16" t="inlineStr">
         <is>
           <t>Recipient(s): Change Requester</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="12" t="inlineStr">
+      <c r="A31" s="13" t="inlineStr">
         <is>
           <t>Workflow diagram</t>
         </is>
@@ -1639,7 +2183,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1667,213 +2211,213 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="21" t="inlineStr">
         <is>
           <t>Proposal</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Stage #</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Stage Name</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>In this variant</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="n">
+      <c r="A5" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>Initiation</t>
         </is>
       </c>
-      <c r="C5" s="11" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="14" t="n">
+      <c r="A6" s="23" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="14" t="inlineStr">
+      <c r="B6" s="23" t="inlineStr">
         <is>
           <t>Evaluation, Design &amp; Analysis</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr">
+      <c r="C6" s="23" t="inlineStr">
         <is>
           <t>Skipped</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="15" t="n">
+      <c r="A7" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="15" t="inlineStr">
+      <c r="B7" s="12" t="inlineStr">
         <is>
           <t>Approval</t>
         </is>
       </c>
-      <c r="C7" s="15" t="inlineStr">
+      <c r="C7" s="12" t="inlineStr">
         <is>
           <t>Yes - approver [TBC]</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="n">
+      <c r="A8" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Implementation</t>
         </is>
       </c>
-      <c r="C8" s="11" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="n">
+      <c r="A9" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>Start Up</t>
         </is>
       </c>
-      <c r="C9" s="11" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="n">
+      <c r="A10" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>Follow Up</t>
         </is>
       </c>
-      <c r="C10" s="11" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="inlineStr">
+      <c r="A12" s="13" t="inlineStr">
         <is>
           <t>Detailed workflow (Intelex workbook format)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="13" t="inlineStr">
+      <c r="A13" s="22" t="inlineStr">
         <is>
           <t>Stage #</t>
         </is>
       </c>
-      <c r="B13" s="13" t="inlineStr">
+      <c r="B13" s="22" t="inlineStr">
         <is>
           <t>Stage Name</t>
         </is>
       </c>
-      <c r="C13" s="13" t="inlineStr">
+      <c r="C13" s="22" t="inlineStr">
         <is>
           <t>Record Status</t>
         </is>
       </c>
-      <c r="D13" s="13" t="inlineStr">
+      <c r="D13" s="22" t="inlineStr">
         <is>
           <t>Stage Owner</t>
         </is>
       </c>
-      <c r="E13" s="13" t="inlineStr">
+      <c r="E13" s="22" t="inlineStr">
         <is>
           <t>Due Date</t>
         </is>
       </c>
-      <c r="F13" s="13" t="inlineStr">
+      <c r="F13" s="22" t="inlineStr">
         <is>
           <t>Workflow Buttons</t>
         </is>
       </c>
-      <c r="G13" s="13" t="inlineStr">
+      <c r="G13" s="22" t="inlineStr">
         <is>
           <t>Workflow Path</t>
         </is>
       </c>
-      <c r="H13" s="13" t="inlineStr">
+      <c r="H13" s="22" t="inlineStr">
         <is>
           <t>Email Template #</t>
         </is>
       </c>
-      <c r="I13" s="13" t="inlineStr">
+      <c r="I13" s="22" t="inlineStr">
         <is>
           <t>Comments</t>
         </is>
       </c>
     </row>
     <row r="14" ht="60" customHeight="1">
-      <c r="A14" s="5" t="n">
+      <c r="A14" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B14" s="16" t="inlineStr">
         <is>
           <t>Initiation</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C14" s="16" t="inlineStr">
         <is>
           <t>Initiation</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D14" s="16" t="inlineStr">
         <is>
           <t>Created By (Field)</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E14" s="16" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="F14" s="16" t="inlineStr">
         <is>
           <t>Submit</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr">
+      <c r="G14" s="16" t="inlineStr">
         <is>
           <t>Emergency Change = Yes: straight to 'Approval'</t>
         </is>
       </c>
-      <c r="H14" s="7" t="inlineStr">
+      <c r="H14" s="18" t="inlineStr">
         <is>
           <t>N01 + N11 [BA]</t>
         </is>
       </c>
-      <c r="I14" s="7" t="inlineStr">
+      <c r="I14" s="18" t="inlineStr">
         <is>
           <t>Recipient(s): Change Requester, MOC Coordinator
 N11 alert to Terminal Manager + Regional HSEC [BA]. Emergency Justification mandatory [BA].</t>
@@ -1881,90 +2425,90 @@
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="6" t="n">
+      <c r="A15" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="B15" s="6" t="inlineStr">
+      <c r="B15" s="17" t="inlineStr">
         <is>
           <t>Evaluation, Design &amp; Analysis</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="C15" s="17" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D15" s="6" t="inlineStr">
+      <c r="D15" s="17" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E15" s="6" t="inlineStr">
+      <c r="E15" s="17" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F15" s="6" t="inlineStr">
+      <c r="F15" s="17" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G15" s="6" t="inlineStr">
+      <c r="G15" s="17" t="inlineStr">
         <is>
           <t>SKIPPED</t>
         </is>
       </c>
-      <c r="H15" s="6" t="inlineStr">
+      <c r="H15" s="17" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I15" s="6" t="inlineStr">
+      <c r="I15" s="17" t="inlineStr">
         <is>
           <t>Retrospective completion of checklist / dossier? [TBC - BRD RULE-B3-14]</t>
         </is>
       </c>
     </row>
     <row r="16" ht="45" customHeight="1">
-      <c r="A16" s="5" t="n">
+      <c r="A16" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B16" s="16" t="inlineStr">
         <is>
           <t>Approval</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C16" s="16" t="inlineStr">
         <is>
           <t>Approval</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="D16" s="16" t="inlineStr">
         <is>
           <t>MOC Coordinator (Role)</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr">
+      <c r="E16" s="18" t="inlineStr">
         <is>
           <t>[TBC] (urgent)</t>
         </is>
       </c>
-      <c r="F16" s="5" t="inlineStr">
+      <c r="F16" s="16" t="inlineStr">
         <is>
           <t>Submit</t>
         </is>
       </c>
-      <c r="G16" s="5" t="inlineStr">
+      <c r="G16" s="16" t="inlineStr">
         <is>
           <t>To 'Implementation'</t>
         </is>
       </c>
-      <c r="H16" s="5" t="inlineStr">
+      <c r="H16" s="16" t="inlineStr">
         <is>
           <t>N01 / N08</t>
         </is>
       </c>
-      <c r="I16" s="7" t="inlineStr">
+      <c r="I16" s="18" t="inlineStr">
         <is>
           <t>Recipient(s): Change Requester
 Approvals by Change Impact (as full flow) or single senior approver? [TBC]</t>
@@ -1972,95 +2516,95 @@
       </c>
     </row>
     <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="5" t="n"/>
-      <c r="B17" s="5" t="n"/>
-      <c r="C17" s="5" t="n"/>
-      <c r="D17" s="5" t="n"/>
-      <c r="E17" s="5" t="n"/>
-      <c r="F17" s="5" t="inlineStr">
+      <c r="A17" s="16" t="n"/>
+      <c r="B17" s="16" t="n"/>
+      <c r="C17" s="16" t="n"/>
+      <c r="D17" s="16" t="n"/>
+      <c r="E17" s="16" t="n"/>
+      <c r="F17" s="16" t="inlineStr">
         <is>
           <t>Roll Back</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr">
+      <c r="G17" s="16" t="inlineStr">
         <is>
           <t>Back to 'Initiation'</t>
         </is>
       </c>
-      <c r="H17" s="5" t="inlineStr">
+      <c r="H17" s="16" t="inlineStr">
         <is>
           <t>N02</t>
         </is>
       </c>
-      <c r="I17" s="5" t="inlineStr">
+      <c r="I17" s="16" t="inlineStr">
         <is>
           <t>Recipient(s): Change Requester</t>
         </is>
       </c>
     </row>
     <row r="18" ht="16" customHeight="1">
-      <c r="A18" s="5" t="n"/>
-      <c r="B18" s="5" t="n"/>
-      <c r="C18" s="5" t="n"/>
-      <c r="D18" s="5" t="n"/>
-      <c r="E18" s="5" t="n"/>
-      <c r="F18" s="5" t="inlineStr">
+      <c r="A18" s="16" t="n"/>
+      <c r="B18" s="16" t="n"/>
+      <c r="C18" s="16" t="n"/>
+      <c r="D18" s="16" t="n"/>
+      <c r="E18" s="16" t="n"/>
+      <c r="F18" s="16" t="inlineStr">
         <is>
           <t>Cancel</t>
         </is>
       </c>
-      <c r="G18" s="5" t="inlineStr"/>
-      <c r="H18" s="5" t="inlineStr">
+      <c r="G18" s="16" t="inlineStr"/>
+      <c r="H18" s="16" t="inlineStr">
         <is>
           <t>N03</t>
         </is>
       </c>
-      <c r="I18" s="5" t="inlineStr">
+      <c r="I18" s="16" t="inlineStr">
         <is>
           <t>Recipient(s): Change Requester</t>
         </is>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="5" t="n">
+      <c r="A19" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B19" s="16" t="inlineStr">
         <is>
           <t>Implementation</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C19" s="16" t="inlineStr">
         <is>
           <t>Implementation</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
+      <c r="D19" s="16" t="inlineStr">
         <is>
           <t>MOC Coordinator (Role)</t>
         </is>
       </c>
-      <c r="E19" s="5" t="inlineStr">
+      <c r="E19" s="16" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="F19" s="5" t="inlineStr">
+      <c r="F19" s="16" t="inlineStr">
         <is>
           <t>Submit</t>
         </is>
       </c>
-      <c r="G19" s="5" t="inlineStr">
+      <c r="G19" s="16" t="inlineStr">
         <is>
           <t>To 'Start Up'</t>
         </is>
       </c>
-      <c r="H19" s="5" t="inlineStr">
+      <c r="H19" s="16" t="inlineStr">
         <is>
           <t>N01</t>
         </is>
       </c>
-      <c r="I19" s="5" t="inlineStr">
+      <c r="I19" s="16" t="inlineStr">
         <is>
           <t>Recipient(s): Change Requester
 Same as full flow.</t>
@@ -2068,95 +2612,95 @@
       </c>
     </row>
     <row r="20" ht="16" customHeight="1">
-      <c r="A20" s="5" t="n"/>
-      <c r="B20" s="5" t="n"/>
-      <c r="C20" s="5" t="n"/>
-      <c r="D20" s="5" t="n"/>
-      <c r="E20" s="5" t="n"/>
-      <c r="F20" s="5" t="inlineStr">
+      <c r="A20" s="16" t="n"/>
+      <c r="B20" s="16" t="n"/>
+      <c r="C20" s="16" t="n"/>
+      <c r="D20" s="16" t="n"/>
+      <c r="E20" s="16" t="n"/>
+      <c r="F20" s="16" t="inlineStr">
         <is>
           <t>Roll Back</t>
         </is>
       </c>
-      <c r="G20" s="5" t="inlineStr">
+      <c r="G20" s="16" t="inlineStr">
         <is>
           <t>Back to 'Approval'</t>
         </is>
       </c>
-      <c r="H20" s="5" t="inlineStr">
+      <c r="H20" s="16" t="inlineStr">
         <is>
           <t>N02</t>
         </is>
       </c>
-      <c r="I20" s="5" t="inlineStr">
+      <c r="I20" s="16" t="inlineStr">
         <is>
           <t>Recipient(s): Change Requester</t>
         </is>
       </c>
     </row>
     <row r="21" ht="16" customHeight="1">
-      <c r="A21" s="5" t="n"/>
-      <c r="B21" s="5" t="n"/>
-      <c r="C21" s="5" t="n"/>
-      <c r="D21" s="5" t="n"/>
-      <c r="E21" s="5" t="n"/>
-      <c r="F21" s="5" t="inlineStr">
+      <c r="A21" s="16" t="n"/>
+      <c r="B21" s="16" t="n"/>
+      <c r="C21" s="16" t="n"/>
+      <c r="D21" s="16" t="n"/>
+      <c r="E21" s="16" t="n"/>
+      <c r="F21" s="16" t="inlineStr">
         <is>
           <t>Cancel</t>
         </is>
       </c>
-      <c r="G21" s="5" t="inlineStr"/>
-      <c r="H21" s="5" t="inlineStr">
+      <c r="G21" s="16" t="inlineStr"/>
+      <c r="H21" s="16" t="inlineStr">
         <is>
           <t>N03</t>
         </is>
       </c>
-      <c r="I21" s="5" t="inlineStr">
+      <c r="I21" s="16" t="inlineStr">
         <is>
           <t>Recipient(s): Change Requester</t>
         </is>
       </c>
     </row>
     <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="5" t="n">
+      <c r="A22" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="B22" s="16" t="inlineStr">
         <is>
           <t>Start Up</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
+      <c r="C22" s="16" t="inlineStr">
         <is>
           <t>Start Up</t>
         </is>
       </c>
-      <c r="D22" s="5" t="inlineStr">
+      <c r="D22" s="16" t="inlineStr">
         <is>
           <t>MOC Coordinator (Role)</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr">
+      <c r="E22" s="16" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="F22" s="5" t="inlineStr">
+      <c r="F22" s="16" t="inlineStr">
         <is>
           <t>Submit</t>
         </is>
       </c>
-      <c r="G22" s="5" t="inlineStr">
+      <c r="G22" s="16" t="inlineStr">
         <is>
           <t>To 'Follow Up'</t>
         </is>
       </c>
-      <c r="H22" s="5" t="inlineStr">
+      <c r="H22" s="16" t="inlineStr">
         <is>
           <t>N01</t>
         </is>
       </c>
-      <c r="I22" s="5" t="inlineStr">
+      <c r="I22" s="16" t="inlineStr">
         <is>
           <t>Recipient(s): Change Requester
 Same as full flow.</t>
@@ -2164,91 +2708,91 @@
       </c>
     </row>
     <row r="23" ht="16" customHeight="1">
-      <c r="A23" s="5" t="n"/>
-      <c r="B23" s="5" t="n"/>
-      <c r="C23" s="5" t="n"/>
-      <c r="D23" s="5" t="n"/>
-      <c r="E23" s="5" t="n"/>
-      <c r="F23" s="5" t="inlineStr">
+      <c r="A23" s="16" t="n"/>
+      <c r="B23" s="16" t="n"/>
+      <c r="C23" s="16" t="n"/>
+      <c r="D23" s="16" t="n"/>
+      <c r="E23" s="16" t="n"/>
+      <c r="F23" s="16" t="inlineStr">
         <is>
           <t>Roll Back</t>
         </is>
       </c>
-      <c r="G23" s="5" t="inlineStr">
+      <c r="G23" s="16" t="inlineStr">
         <is>
           <t>Back to 'Implementation'</t>
         </is>
       </c>
-      <c r="H23" s="5" t="inlineStr">
+      <c r="H23" s="16" t="inlineStr">
         <is>
           <t>N02</t>
         </is>
       </c>
-      <c r="I23" s="5" t="inlineStr">
+      <c r="I23" s="16" t="inlineStr">
         <is>
           <t>Recipient(s): Change Requester</t>
         </is>
       </c>
     </row>
     <row r="24" ht="16" customHeight="1">
-      <c r="A24" s="5" t="n"/>
-      <c r="B24" s="5" t="n"/>
-      <c r="C24" s="5" t="n"/>
-      <c r="D24" s="5" t="n"/>
-      <c r="E24" s="5" t="n"/>
-      <c r="F24" s="5" t="inlineStr">
+      <c r="A24" s="16" t="n"/>
+      <c r="B24" s="16" t="n"/>
+      <c r="C24" s="16" t="n"/>
+      <c r="D24" s="16" t="n"/>
+      <c r="E24" s="16" t="n"/>
+      <c r="F24" s="16" t="inlineStr">
         <is>
           <t>Cancel</t>
         </is>
       </c>
-      <c r="G24" s="5" t="inlineStr"/>
-      <c r="H24" s="5" t="inlineStr">
+      <c r="G24" s="16" t="inlineStr"/>
+      <c r="H24" s="16" t="inlineStr">
         <is>
           <t>N03</t>
         </is>
       </c>
-      <c r="I24" s="5" t="inlineStr">
+      <c r="I24" s="16" t="inlineStr">
         <is>
           <t>Recipient(s): Change Requester</t>
         </is>
       </c>
     </row>
     <row r="25" ht="45" customHeight="1">
-      <c r="A25" s="5" t="n">
+      <c r="A25" s="16" t="n">
         <v>6</v>
       </c>
-      <c r="B25" s="5" t="inlineStr">
+      <c r="B25" s="16" t="inlineStr">
         <is>
           <t>Follow Up</t>
         </is>
       </c>
-      <c r="C25" s="5" t="inlineStr">
+      <c r="C25" s="16" t="inlineStr">
         <is>
           <t>Follow Up</t>
         </is>
       </c>
-      <c r="D25" s="5" t="inlineStr">
+      <c r="D25" s="16" t="inlineStr">
         <is>
           <t>MOC Coordinator (Role)</t>
         </is>
       </c>
-      <c r="E25" s="5" t="inlineStr">
+      <c r="E25" s="16" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="F25" s="5" t="inlineStr">
+      <c r="F25" s="16" t="inlineStr">
         <is>
           <t>Close</t>
         </is>
       </c>
-      <c r="G25" s="5" t="inlineStr"/>
-      <c r="H25" s="5" t="inlineStr">
+      <c r="G25" s="16" t="inlineStr"/>
+      <c r="H25" s="16" t="inlineStr">
         <is>
           <t>N04</t>
         </is>
       </c>
-      <c r="I25" s="7" t="inlineStr">
+      <c r="I25" s="18" t="inlineStr">
         <is>
           <t>Recipient(s): Change Requester
 Close only when the emergency dossier is regularised [TBC].</t>
@@ -2256,57 +2800,57 @@
       </c>
     </row>
     <row r="26" ht="16" customHeight="1">
-      <c r="A26" s="5" t="n"/>
-      <c r="B26" s="5" t="n"/>
-      <c r="C26" s="5" t="n"/>
-      <c r="D26" s="5" t="n"/>
-      <c r="E26" s="5" t="n"/>
-      <c r="F26" s="5" t="inlineStr">
+      <c r="A26" s="16" t="n"/>
+      <c r="B26" s="16" t="n"/>
+      <c r="C26" s="16" t="n"/>
+      <c r="D26" s="16" t="n"/>
+      <c r="E26" s="16" t="n"/>
+      <c r="F26" s="16" t="inlineStr">
         <is>
           <t>Roll Back</t>
         </is>
       </c>
-      <c r="G26" s="5" t="inlineStr">
+      <c r="G26" s="16" t="inlineStr">
         <is>
           <t>Back to 'Start Up'</t>
         </is>
       </c>
-      <c r="H26" s="5" t="inlineStr">
+      <c r="H26" s="16" t="inlineStr">
         <is>
           <t>N02</t>
         </is>
       </c>
-      <c r="I26" s="5" t="inlineStr">
+      <c r="I26" s="16" t="inlineStr">
         <is>
           <t>Recipient(s): Change Requester</t>
         </is>
       </c>
     </row>
     <row r="27" ht="16" customHeight="1">
-      <c r="A27" s="5" t="n"/>
-      <c r="B27" s="5" t="n"/>
-      <c r="C27" s="5" t="n"/>
-      <c r="D27" s="5" t="n"/>
-      <c r="E27" s="5" t="n"/>
-      <c r="F27" s="5" t="inlineStr">
+      <c r="A27" s="16" t="n"/>
+      <c r="B27" s="16" t="n"/>
+      <c r="C27" s="16" t="n"/>
+      <c r="D27" s="16" t="n"/>
+      <c r="E27" s="16" t="n"/>
+      <c r="F27" s="16" t="inlineStr">
         <is>
           <t>Cancel</t>
         </is>
       </c>
-      <c r="G27" s="5" t="inlineStr"/>
-      <c r="H27" s="5" t="inlineStr">
+      <c r="G27" s="16" t="inlineStr"/>
+      <c r="H27" s="16" t="inlineStr">
         <is>
           <t>N03</t>
         </is>
       </c>
-      <c r="I27" s="5" t="inlineStr">
+      <c r="I27" s="16" t="inlineStr">
         <is>
           <t>Recipient(s): Change Requester</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="12" t="inlineStr">
+      <c r="A29" s="13" t="inlineStr">
         <is>
           <t>Workflow diagram</t>
         </is>
@@ -2321,7 +2865,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2349,213 +2893,213 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="21" t="inlineStr">
         <is>
           <t>Proposal</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Stage #</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Stage Name</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>In this variant</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="n">
+      <c r="A5" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>Initiation</t>
         </is>
       </c>
-      <c r="C5" s="11" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="n">
+      <c r="A6" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="11" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Evaluation, Design &amp; Analysis</t>
         </is>
       </c>
-      <c r="C6" s="11" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>Yes - no checklist</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="n">
+      <c r="A7" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Approval</t>
         </is>
       </c>
-      <c r="C7" s="11" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="n">
+      <c r="A8" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Implementation</t>
         </is>
       </c>
-      <c r="C8" s="11" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="15" t="n">
+      <c r="A9" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="15" t="inlineStr">
+      <c r="B9" s="12" t="inlineStr">
         <is>
           <t>Start Up</t>
         </is>
       </c>
-      <c r="C9" s="15" t="inlineStr">
+      <c r="C9" s="12" t="inlineStr">
         <is>
           <t>Yes - applicable? [TBC]</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="n">
+      <c r="A10" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>Follow Up</t>
         </is>
       </c>
-      <c r="C10" s="11" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="inlineStr">
+      <c r="A12" s="13" t="inlineStr">
         <is>
           <t>Detailed workflow (Intelex workbook format)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="13" t="inlineStr">
+      <c r="A13" s="22" t="inlineStr">
         <is>
           <t>Stage #</t>
         </is>
       </c>
-      <c r="B13" s="13" t="inlineStr">
+      <c r="B13" s="22" t="inlineStr">
         <is>
           <t>Stage Name</t>
         </is>
       </c>
-      <c r="C13" s="13" t="inlineStr">
+      <c r="C13" s="22" t="inlineStr">
         <is>
           <t>Record Status</t>
         </is>
       </c>
-      <c r="D13" s="13" t="inlineStr">
+      <c r="D13" s="22" t="inlineStr">
         <is>
           <t>Stage Owner</t>
         </is>
       </c>
-      <c r="E13" s="13" t="inlineStr">
+      <c r="E13" s="22" t="inlineStr">
         <is>
           <t>Due Date</t>
         </is>
       </c>
-      <c r="F13" s="13" t="inlineStr">
+      <c r="F13" s="22" t="inlineStr">
         <is>
           <t>Workflow Buttons</t>
         </is>
       </c>
-      <c r="G13" s="13" t="inlineStr">
+      <c r="G13" s="22" t="inlineStr">
         <is>
           <t>Workflow Path</t>
         </is>
       </c>
-      <c r="H13" s="13" t="inlineStr">
+      <c r="H13" s="22" t="inlineStr">
         <is>
           <t>Email Template #</t>
         </is>
       </c>
-      <c r="I13" s="13" t="inlineStr">
+      <c r="I13" s="22" t="inlineStr">
         <is>
           <t>Comments</t>
         </is>
       </c>
     </row>
     <row r="14" ht="45" customHeight="1">
-      <c r="A14" s="5" t="n">
+      <c r="A14" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B14" s="16" t="inlineStr">
         <is>
           <t>Initiation</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C14" s="16" t="inlineStr">
         <is>
           <t>Initiation</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D14" s="16" t="inlineStr">
         <is>
           <t>Created By (Field)</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E14" s="16" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="F14" s="16" t="inlineStr">
         <is>
           <t>Submit</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr">
+      <c r="G14" s="16" t="inlineStr">
         <is>
           <t>To 'Evaluation, Design &amp; Analysis'</t>
         </is>
       </c>
-      <c r="H14" s="5" t="inlineStr">
+      <c r="H14" s="16" t="inlineStr">
         <is>
           <t>N01</t>
         </is>
       </c>
-      <c r="I14" s="5" t="inlineStr">
+      <c r="I14" s="16" t="inlineStr">
         <is>
           <t>Recipient(s): Change Requester
 Simple Change = Yes (IT / organisational changes).</t>
@@ -2563,45 +3107,45 @@
       </c>
     </row>
     <row r="15" ht="60" customHeight="1">
-      <c r="A15" s="5" t="n">
+      <c r="A15" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B15" s="16" t="inlineStr">
         <is>
           <t>Evaluation, Design &amp; Analysis</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C15" s="16" t="inlineStr">
         <is>
           <t>Evaluation, Design &amp; Analysis</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D15" s="16" t="inlineStr">
         <is>
           <t>MOC Coordinator (Role)</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="E15" s="16" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="F15" s="16" t="inlineStr">
         <is>
           <t>Submit</t>
         </is>
       </c>
-      <c r="G15" s="5" t="inlineStr">
+      <c r="G15" s="16" t="inlineStr">
         <is>
           <t>To 'Approval'</t>
         </is>
       </c>
-      <c r="H15" s="5" t="inlineStr">
+      <c r="H15" s="16" t="inlineStr">
         <is>
           <t>N01</t>
         </is>
       </c>
-      <c r="I15" s="7" t="inlineStr">
+      <c r="I15" s="18" t="inlineStr">
         <is>
           <t>Recipient(s): Change Requester
 NO checklist generated. Tasks + D&amp;A questions - which apply? [TBC]. 'Different process review' [TBC].</t>
@@ -2609,95 +3153,95 @@
       </c>
     </row>
     <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="5" t="n"/>
-      <c r="B16" s="5" t="n"/>
-      <c r="C16" s="5" t="n"/>
-      <c r="D16" s="5" t="n"/>
-      <c r="E16" s="5" t="n"/>
-      <c r="F16" s="5" t="inlineStr">
+      <c r="A16" s="16" t="n"/>
+      <c r="B16" s="16" t="n"/>
+      <c r="C16" s="16" t="n"/>
+      <c r="D16" s="16" t="n"/>
+      <c r="E16" s="16" t="n"/>
+      <c r="F16" s="16" t="inlineStr">
         <is>
           <t>Roll Back</t>
         </is>
       </c>
-      <c r="G16" s="5" t="inlineStr">
+      <c r="G16" s="16" t="inlineStr">
         <is>
           <t>Back to 'Initiation'</t>
         </is>
       </c>
-      <c r="H16" s="5" t="inlineStr">
+      <c r="H16" s="16" t="inlineStr">
         <is>
           <t>N02</t>
         </is>
       </c>
-      <c r="I16" s="5" t="inlineStr">
+      <c r="I16" s="16" t="inlineStr">
         <is>
           <t>Recipient(s): Change Requester</t>
         </is>
       </c>
     </row>
     <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="5" t="n"/>
-      <c r="B17" s="5" t="n"/>
-      <c r="C17" s="5" t="n"/>
-      <c r="D17" s="5" t="n"/>
-      <c r="E17" s="5" t="n"/>
-      <c r="F17" s="5" t="inlineStr">
+      <c r="A17" s="16" t="n"/>
+      <c r="B17" s="16" t="n"/>
+      <c r="C17" s="16" t="n"/>
+      <c r="D17" s="16" t="n"/>
+      <c r="E17" s="16" t="n"/>
+      <c r="F17" s="16" t="inlineStr">
         <is>
           <t>Cancel</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr"/>
-      <c r="H17" s="5" t="inlineStr">
+      <c r="G17" s="16" t="inlineStr"/>
+      <c r="H17" s="16" t="inlineStr">
         <is>
           <t>N03</t>
         </is>
       </c>
-      <c r="I17" s="5" t="inlineStr">
+      <c r="I17" s="16" t="inlineStr">
         <is>
           <t>Recipient(s): Change Requester</t>
         </is>
       </c>
     </row>
     <row r="18" ht="45" customHeight="1">
-      <c r="A18" s="5" t="n">
+      <c r="A18" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B18" s="16" t="inlineStr">
         <is>
           <t>Approval</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="C18" s="16" t="inlineStr">
         <is>
           <t>Approval</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="D18" s="16" t="inlineStr">
         <is>
           <t>MOC Coordinator (Role)</t>
         </is>
       </c>
-      <c r="E18" s="5" t="inlineStr">
+      <c r="E18" s="16" t="inlineStr">
         <is>
           <t>7 days</t>
         </is>
       </c>
-      <c r="F18" s="5" t="inlineStr">
+      <c r="F18" s="16" t="inlineStr">
         <is>
           <t>Submit</t>
         </is>
       </c>
-      <c r="G18" s="5" t="inlineStr">
+      <c r="G18" s="16" t="inlineStr">
         <is>
           <t>To 'Implementation'</t>
         </is>
       </c>
-      <c r="H18" s="5" t="inlineStr">
+      <c r="H18" s="16" t="inlineStr">
         <is>
           <t>N01 / N08</t>
         </is>
       </c>
-      <c r="I18" s="5" t="inlineStr">
+      <c r="I18" s="16" t="inlineStr">
         <is>
           <t>Recipient(s): Change Requester
 Approvals by Change Impact, sequential (as full flow).</t>
@@ -2705,95 +3249,95 @@
       </c>
     </row>
     <row r="19" ht="16" customHeight="1">
-      <c r="A19" s="5" t="n"/>
-      <c r="B19" s="5" t="n"/>
-      <c r="C19" s="5" t="n"/>
-      <c r="D19" s="5" t="n"/>
-      <c r="E19" s="5" t="n"/>
-      <c r="F19" s="5" t="inlineStr">
+      <c r="A19" s="16" t="n"/>
+      <c r="B19" s="16" t="n"/>
+      <c r="C19" s="16" t="n"/>
+      <c r="D19" s="16" t="n"/>
+      <c r="E19" s="16" t="n"/>
+      <c r="F19" s="16" t="inlineStr">
         <is>
           <t>Roll Back</t>
         </is>
       </c>
-      <c r="G19" s="5" t="inlineStr">
+      <c r="G19" s="16" t="inlineStr">
         <is>
           <t>Back to 'Evaluation, Design &amp; Analysis'</t>
         </is>
       </c>
-      <c r="H19" s="5" t="inlineStr">
+      <c r="H19" s="16" t="inlineStr">
         <is>
           <t>N02</t>
         </is>
       </c>
-      <c r="I19" s="5" t="inlineStr">
+      <c r="I19" s="16" t="inlineStr">
         <is>
           <t>Recipient(s): Change Requester</t>
         </is>
       </c>
     </row>
     <row r="20" ht="16" customHeight="1">
-      <c r="A20" s="5" t="n"/>
-      <c r="B20" s="5" t="n"/>
-      <c r="C20" s="5" t="n"/>
-      <c r="D20" s="5" t="n"/>
-      <c r="E20" s="5" t="n"/>
-      <c r="F20" s="5" t="inlineStr">
+      <c r="A20" s="16" t="n"/>
+      <c r="B20" s="16" t="n"/>
+      <c r="C20" s="16" t="n"/>
+      <c r="D20" s="16" t="n"/>
+      <c r="E20" s="16" t="n"/>
+      <c r="F20" s="16" t="inlineStr">
         <is>
           <t>Cancel</t>
         </is>
       </c>
-      <c r="G20" s="5" t="inlineStr"/>
-      <c r="H20" s="5" t="inlineStr">
+      <c r="G20" s="16" t="inlineStr"/>
+      <c r="H20" s="16" t="inlineStr">
         <is>
           <t>N03</t>
         </is>
       </c>
-      <c r="I20" s="5" t="inlineStr">
+      <c r="I20" s="16" t="inlineStr">
         <is>
           <t>Recipient(s): Change Requester</t>
         </is>
       </c>
     </row>
     <row r="21" ht="45" customHeight="1">
-      <c r="A21" s="5" t="n">
+      <c r="A21" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="B21" s="16" t="inlineStr">
         <is>
           <t>Implementation</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="C21" s="16" t="inlineStr">
         <is>
           <t>Implementation</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="D21" s="16" t="inlineStr">
         <is>
           <t>MOC Coordinator (Role)</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr">
+      <c r="E21" s="16" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="F21" s="5" t="inlineStr">
+      <c r="F21" s="16" t="inlineStr">
         <is>
           <t>Submit</t>
         </is>
       </c>
-      <c r="G21" s="5" t="inlineStr">
+      <c r="G21" s="16" t="inlineStr">
         <is>
           <t>To 'Start Up'</t>
         </is>
       </c>
-      <c r="H21" s="5" t="inlineStr">
+      <c r="H21" s="16" t="inlineStr">
         <is>
           <t>N01</t>
         </is>
       </c>
-      <c r="I21" s="7" t="inlineStr">
+      <c r="I21" s="18" t="inlineStr">
         <is>
           <t>Recipient(s): Change Requester
 PSSR applicable? [TBC]. Training + communication.</t>
@@ -2801,95 +3345,95 @@
       </c>
     </row>
     <row r="22" ht="16" customHeight="1">
-      <c r="A22" s="5" t="n"/>
-      <c r="B22" s="5" t="n"/>
-      <c r="C22" s="5" t="n"/>
-      <c r="D22" s="5" t="n"/>
-      <c r="E22" s="5" t="n"/>
-      <c r="F22" s="5" t="inlineStr">
+      <c r="A22" s="16" t="n"/>
+      <c r="B22" s="16" t="n"/>
+      <c r="C22" s="16" t="n"/>
+      <c r="D22" s="16" t="n"/>
+      <c r="E22" s="16" t="n"/>
+      <c r="F22" s="16" t="inlineStr">
         <is>
           <t>Roll Back</t>
         </is>
       </c>
-      <c r="G22" s="5" t="inlineStr">
+      <c r="G22" s="16" t="inlineStr">
         <is>
           <t>Back to 'Approval'</t>
         </is>
       </c>
-      <c r="H22" s="5" t="inlineStr">
+      <c r="H22" s="16" t="inlineStr">
         <is>
           <t>N02</t>
         </is>
       </c>
-      <c r="I22" s="5" t="inlineStr">
+      <c r="I22" s="16" t="inlineStr">
         <is>
           <t>Recipient(s): Change Requester</t>
         </is>
       </c>
     </row>
     <row r="23" ht="16" customHeight="1">
-      <c r="A23" s="5" t="n"/>
-      <c r="B23" s="5" t="n"/>
-      <c r="C23" s="5" t="n"/>
-      <c r="D23" s="5" t="n"/>
-      <c r="E23" s="5" t="n"/>
-      <c r="F23" s="5" t="inlineStr">
+      <c r="A23" s="16" t="n"/>
+      <c r="B23" s="16" t="n"/>
+      <c r="C23" s="16" t="n"/>
+      <c r="D23" s="16" t="n"/>
+      <c r="E23" s="16" t="n"/>
+      <c r="F23" s="16" t="inlineStr">
         <is>
           <t>Cancel</t>
         </is>
       </c>
-      <c r="G23" s="5" t="inlineStr"/>
-      <c r="H23" s="5" t="inlineStr">
+      <c r="G23" s="16" t="inlineStr"/>
+      <c r="H23" s="16" t="inlineStr">
         <is>
           <t>N03</t>
         </is>
       </c>
-      <c r="I23" s="5" t="inlineStr">
+      <c r="I23" s="16" t="inlineStr">
         <is>
           <t>Recipient(s): Change Requester</t>
         </is>
       </c>
     </row>
     <row r="24" ht="45" customHeight="1">
-      <c r="A24" s="5" t="n">
+      <c r="A24" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="B24" s="5" t="inlineStr">
+      <c r="B24" s="16" t="inlineStr">
         <is>
           <t>Start Up</t>
         </is>
       </c>
-      <c r="C24" s="5" t="inlineStr">
+      <c r="C24" s="16" t="inlineStr">
         <is>
           <t>Start Up</t>
         </is>
       </c>
-      <c r="D24" s="5" t="inlineStr">
+      <c r="D24" s="16" t="inlineStr">
         <is>
           <t>MOC Coordinator (Role)</t>
         </is>
       </c>
-      <c r="E24" s="5" t="inlineStr">
+      <c r="E24" s="16" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="F24" s="5" t="inlineStr">
+      <c r="F24" s="16" t="inlineStr">
         <is>
           <t>Submit</t>
         </is>
       </c>
-      <c r="G24" s="5" t="inlineStr">
+      <c r="G24" s="16" t="inlineStr">
         <is>
           <t>To 'Follow Up'</t>
         </is>
       </c>
-      <c r="H24" s="5" t="inlineStr">
+      <c r="H24" s="16" t="inlineStr">
         <is>
           <t>N01</t>
         </is>
       </c>
-      <c r="I24" s="7" t="inlineStr">
+      <c r="I24" s="18" t="inlineStr">
         <is>
           <t>Recipient(s): Change Requester
 Applicable to IT / Org changes? [TBC]</t>
@@ -2897,91 +3441,91 @@
       </c>
     </row>
     <row r="25" ht="16" customHeight="1">
-      <c r="A25" s="5" t="n"/>
-      <c r="B25" s="5" t="n"/>
-      <c r="C25" s="5" t="n"/>
-      <c r="D25" s="5" t="n"/>
-      <c r="E25" s="5" t="n"/>
-      <c r="F25" s="5" t="inlineStr">
+      <c r="A25" s="16" t="n"/>
+      <c r="B25" s="16" t="n"/>
+      <c r="C25" s="16" t="n"/>
+      <c r="D25" s="16" t="n"/>
+      <c r="E25" s="16" t="n"/>
+      <c r="F25" s="16" t="inlineStr">
         <is>
           <t>Roll Back</t>
         </is>
       </c>
-      <c r="G25" s="5" t="inlineStr">
+      <c r="G25" s="16" t="inlineStr">
         <is>
           <t>Back to 'Implementation'</t>
         </is>
       </c>
-      <c r="H25" s="5" t="inlineStr">
+      <c r="H25" s="16" t="inlineStr">
         <is>
           <t>N02</t>
         </is>
       </c>
-      <c r="I25" s="5" t="inlineStr">
+      <c r="I25" s="16" t="inlineStr">
         <is>
           <t>Recipient(s): Change Requester</t>
         </is>
       </c>
     </row>
     <row r="26" ht="16" customHeight="1">
-      <c r="A26" s="5" t="n"/>
-      <c r="B26" s="5" t="n"/>
-      <c r="C26" s="5" t="n"/>
-      <c r="D26" s="5" t="n"/>
-      <c r="E26" s="5" t="n"/>
-      <c r="F26" s="5" t="inlineStr">
+      <c r="A26" s="16" t="n"/>
+      <c r="B26" s="16" t="n"/>
+      <c r="C26" s="16" t="n"/>
+      <c r="D26" s="16" t="n"/>
+      <c r="E26" s="16" t="n"/>
+      <c r="F26" s="16" t="inlineStr">
         <is>
           <t>Cancel</t>
         </is>
       </c>
-      <c r="G26" s="5" t="inlineStr"/>
-      <c r="H26" s="5" t="inlineStr">
+      <c r="G26" s="16" t="inlineStr"/>
+      <c r="H26" s="16" t="inlineStr">
         <is>
           <t>N03</t>
         </is>
       </c>
-      <c r="I26" s="5" t="inlineStr">
+      <c r="I26" s="16" t="inlineStr">
         <is>
           <t>Recipient(s): Change Requester</t>
         </is>
       </c>
     </row>
     <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="5" t="n">
+      <c r="A27" s="16" t="n">
         <v>6</v>
       </c>
-      <c r="B27" s="5" t="inlineStr">
+      <c r="B27" s="16" t="inlineStr">
         <is>
           <t>Follow Up</t>
         </is>
       </c>
-      <c r="C27" s="5" t="inlineStr">
+      <c r="C27" s="16" t="inlineStr">
         <is>
           <t>Follow Up</t>
         </is>
       </c>
-      <c r="D27" s="5" t="inlineStr">
+      <c r="D27" s="16" t="inlineStr">
         <is>
           <t>MOC Coordinator (Role)</t>
         </is>
       </c>
-      <c r="E27" s="5" t="inlineStr">
+      <c r="E27" s="16" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="F27" s="5" t="inlineStr">
+      <c r="F27" s="16" t="inlineStr">
         <is>
           <t>Close</t>
         </is>
       </c>
-      <c r="G27" s="5" t="inlineStr"/>
-      <c r="H27" s="5" t="inlineStr">
+      <c r="G27" s="16" t="inlineStr"/>
+      <c r="H27" s="16" t="inlineStr">
         <is>
           <t>N04</t>
         </is>
       </c>
-      <c r="I27" s="5" t="inlineStr">
+      <c r="I27" s="16" t="inlineStr">
         <is>
           <t>Recipient(s): Change Requester
 Lessons Learnt.</t>
@@ -2989,57 +3533,57 @@
       </c>
     </row>
     <row r="28" ht="16" customHeight="1">
-      <c r="A28" s="5" t="n"/>
-      <c r="B28" s="5" t="n"/>
-      <c r="C28" s="5" t="n"/>
-      <c r="D28" s="5" t="n"/>
-      <c r="E28" s="5" t="n"/>
-      <c r="F28" s="5" t="inlineStr">
+      <c r="A28" s="16" t="n"/>
+      <c r="B28" s="16" t="n"/>
+      <c r="C28" s="16" t="n"/>
+      <c r="D28" s="16" t="n"/>
+      <c r="E28" s="16" t="n"/>
+      <c r="F28" s="16" t="inlineStr">
         <is>
           <t>Roll Back</t>
         </is>
       </c>
-      <c r="G28" s="5" t="inlineStr">
+      <c r="G28" s="16" t="inlineStr">
         <is>
           <t>Back to 'Start Up'</t>
         </is>
       </c>
-      <c r="H28" s="5" t="inlineStr">
+      <c r="H28" s="16" t="inlineStr">
         <is>
           <t>N02</t>
         </is>
       </c>
-      <c r="I28" s="5" t="inlineStr">
+      <c r="I28" s="16" t="inlineStr">
         <is>
           <t>Recipient(s): Change Requester</t>
         </is>
       </c>
     </row>
     <row r="29" ht="16" customHeight="1">
-      <c r="A29" s="5" t="n"/>
-      <c r="B29" s="5" t="n"/>
-      <c r="C29" s="5" t="n"/>
-      <c r="D29" s="5" t="n"/>
-      <c r="E29" s="5" t="n"/>
-      <c r="F29" s="5" t="inlineStr">
+      <c r="A29" s="16" t="n"/>
+      <c r="B29" s="16" t="n"/>
+      <c r="C29" s="16" t="n"/>
+      <c r="D29" s="16" t="n"/>
+      <c r="E29" s="16" t="n"/>
+      <c r="F29" s="16" t="inlineStr">
         <is>
           <t>Cancel</t>
         </is>
       </c>
-      <c r="G29" s="5" t="inlineStr"/>
-      <c r="H29" s="5" t="inlineStr">
+      <c r="G29" s="16" t="inlineStr"/>
+      <c r="H29" s="16" t="inlineStr">
         <is>
           <t>N03</t>
         </is>
       </c>
-      <c r="I29" s="5" t="inlineStr">
+      <c r="I29" s="16" t="inlineStr">
         <is>
           <t>Recipient(s): Change Requester</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="12" t="inlineStr">
+      <c r="A31" s="13" t="inlineStr">
         <is>
           <t>Workflow diagram</t>
         </is>

</xml_diff>

<commit_message>
Add Sam Rev2 proposal mapped onto the 7 OOTB stages to comparison sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018d6Sqji3PhM1w1Xd54RvCw
</commit_message>
<xml_diff>
--- a/docs/moc/Impala - MOC Workflow Variants (Full - Emergency - Simple).xlsx
+++ b/docs/moc/Impala - MOC Workflow Variants (Full - Emergency - Simple).xlsx
@@ -1265,7 +1265,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1748,22 +1748,267 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="19" t="inlineStr">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Proposal on OOTB stages (Sam Rev2 intent, Intelex 7 stages kept)</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="n"/>
+      <c r="C26" s="4" t="n"/>
+      <c r="D26" s="4" t="n"/>
+      <c r="E26" s="4" t="n"/>
+    </row>
+    <row r="27" ht="46" customHeight="1">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Stage #</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Stage Name (OOTB)</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>Simple
+(Simple Change = Yes)</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>Emergency
+(Emergency Change = Yes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>Initiation</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>Pre-Approval → 'Coordinator Review'</t>
+        </is>
+      </c>
+      <c r="C29" s="18" t="inlineStr">
+        <is>
+          <t>✔ one click</t>
+        </is>
+      </c>
+      <c r="D29" s="18" t="inlineStr">
+        <is>
+          <t>✔ one click</t>
+        </is>
+      </c>
+      <c r="E29" s="18" t="inlineStr">
+        <is>
+          <t>✔ one click</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>Evaluation (checklist + tasks)</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="D30" s="18" t="inlineStr">
+        <is>
+          <t>✔ no checklist</t>
+        </is>
+      </c>
+      <c r="E30" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>Design &amp; Analysis + mandated approvals</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="E31" s="18" t="inlineStr">
+        <is>
+          <t>✔ approvals</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>Implementation</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="D32" s="7" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="E32" s="7" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>Start Up</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>Follow Up</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="E34" s="7" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="12" t="n"/>
+      <c r="B35" s="13" t="inlineStr">
+        <is>
+          <t>Path (stage #)</t>
+        </is>
+      </c>
+      <c r="C35" s="14" t="inlineStr">
+        <is>
+          <t>1-2-3-4-5-6-7</t>
+        </is>
+      </c>
+      <c r="D35" s="14" t="inlineStr">
+        <is>
+          <t>1-2-3-4-5-6-7</t>
+        </is>
+      </c>
+      <c r="E35" s="14" t="inlineStr">
+        <is>
+          <t>1-2-4-5-6-7</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Sam's 'Evaluation, D&amp;A' = OOTB Evaluation (checklist) + Design &amp; Analysis (questions); Sam's 'Approval' = mandated approvals in Design &amp; Analysis. Emergency = OOTB emergency path (skips Evaluation). Simple keeps all stages: only change vs OOTB = switch off the Replacement in Kind skip path [Intelex to confirm].</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="19" t="inlineStr">
         <is>
           <t>Legend:</t>
         </is>
       </c>
-      <c r="B26" s="7" t="inlineStr">
+      <c r="B38" s="7" t="inlineStr">
         <is>
           <t>✔ stage applies</t>
         </is>
       </c>
-      <c r="C26" s="10" t="inlineStr">
+      <c r="C38" s="10" t="inlineStr">
         <is>
           <t>— stage skipped</t>
         </is>
       </c>
-      <c r="D26" s="18" t="inlineStr">
+      <c r="D38" s="18" t="inlineStr">
         <is>
           <t>applies with differences</t>
         </is>

</xml_diff>